<commit_message>
Stage 8 fixes: G-008
</commit_message>
<xml_diff>
--- a/output/heldback_firm_G/OsterquillData/Studies/OT-10-S0019/Raw_Observations/Animal_Room/NM31_DRF_041210_OBSERVATIONS.xlsx
+++ b/output/heldback_firm_G/OsterquillData/Studies/OT-10-S0019/Raw_Observations/Animal_Room/NM31_DRF_041210_OBSERVATIONS.xlsx
@@ -189,7 +189,7 @@
   <commentList>
     <comment ref="C4" authorId="0" shapeId="0">
       <text>
-        <t>Stock units were µM on the analytical certificate and nM on the working sheet. Left as received; the conversion is in the dose-lot reconciliation.</t>
+        <t>Delivered dose requires concentration, administration volume, body weight and any stock-unit conversion from the group-linked preparation record. Those source records are unavailable here; no concentration or reconciliation result is inferred.</t>
       </text>
     </comment>
   </commentList>
@@ -204,7 +204,7 @@
   <commentList>
     <comment ref="A2" authorId="0" shapeId="0">
       <text>
-        <t>Cards are complete for the 3M/3F groups. Cross-check against the DRF table is still to be done for the top dose.</t>
+        <t>Top-dose/card reconciliation cannot be established from the group table alone. Source cards are unavailable in this workbook; group findings remain distinct from individual observations.</t>
       </text>
     </comment>
   </commentList>
@@ -590,7 +590,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Animals held after final dose for observation only; no recovery dosing</t>
+          <t>Individual recovery source records unavailable here; no animal-specific recovery conclusion is recorded.</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -739,29 +739,29 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Dose lot records. Concentrations in mg/mL on the current template; vehicle-only lots logged as mg/ml on the legacy sheet.</t>
+          <t>Dose-lot traceability: the DRF table reports delivered dose in mg/kg/day, not formulation concentration.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Lot</t>
+          <t>DRF group</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Date prepared</t>
+          <t>Dose-lot link</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Concentration</t>
+          <t>Administration volume / preparation</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Reconciled by</t>
+          <t>Conversion / reconciliation</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -773,108 +773,120 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>DL-1</t>
+          <t>Vehicle group</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>02/12/2010</t>
+          <t>OQ/2010/000311: group-specific preparation source; lot identifier unavailable</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>per table</t>
+          <t>Group administration-volume and preparation record unavailable</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Rebecca Hawkins</t>
+          <t>Delivered-dose calculation and signed reconciliation source unavailable</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Not independently reconciled here</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>DL-2</t>
+          <t>Low-dose group</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>02/12/2010</t>
+          <t>OQ/2010/000311: group-specific preparation source; lot identifier unavailable</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>µM stock, see note</t>
+          <t>Group administration-volume and preparation record unavailable</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Rebecca Hawkins</t>
+          <t>Delivered-dose calculation and signed reconciliation source unavailable</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Not independently reconciled here</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>DL-3</t>
+          <t>Intermediate-dose group</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>02/19/2010</t>
+          <t>OQ/2010/000311: group-specific preparation source; lot identifier unavailable</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>nM working stock, see note</t>
+          <t>Group administration-volume and preparation record unavailable</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Rebecca Hawkins</t>
+          <t>Delivered-dose calculation and signed reconciliation source unavailable</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Reconciled</t>
+          <t>Not independently reconciled here</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>DL-4</t>
+          <t>Top-dose group</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>02/19/2010</t>
+          <t>OQ/2010/000311: group-specific preparation source; lot identifier unavailable</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>mg/ml</t>
+          <t>Group administration-volume and preparation record unavailable</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Rebecca Hawkins</t>
+          <t>Delivered-dose calculation and signed reconciliation source unavailable</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Reconciled 02/22/2010</t>
+          <t>Not independently reconciled here</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Source units</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Preparation templates use mg/mL or mg/ml; analytical stock labels may use µM or nM. Unit labels are retained as source texture, not concentration results.</t>
         </is>
       </c>
     </row>
@@ -903,7 +915,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Seven-day rat dose-range finding. Clinical observations and body-weight change, individual animal identifiers retained on the animal cards.</t>
+          <t>Seven-day rat dose-range finding: group-level clinical observations and body-weight changes only. Individual-animal identifiers and welfare intervention details require the group-linked animal cards under OQ/2010/000311, unavailable here.</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1043,115 +1055,41 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Recovery observations. Animals held without dosing for observation; findings recorded on the animal cards.</t>
+          <t>Recovery source-record disposition</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Animal</t>
+          <t>Reference</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Sex</t>
+          <t>Dose-group / animal linkage</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Day observed</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
           <t>Finding</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Initials</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>R-01</t>
+          <t>OQ/2010/000311: recovery animal cards</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>Individual identifiers and originating dose groups unavailable</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Day 8</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>No change from dosing period</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>RH</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>R-02</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Day 8</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Body weight recovery noted</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>RH</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>R-03</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Day 9</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Clinical signs resolved</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>VB</t>
+          <t>Recovery findings not transcribed; no supported individual outcome here</t>
         </is>
       </c>
     </row>
@@ -1167,23 +1105,115 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Animal card cross-check. Each card number matched to the observation sheet. Cards retained at the archive per SOP OQ-QA-014.</t>
+          <t>Animal-card linkage and archive limitation</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Card check by Kenji Morita, 04/08/2010. Two cards need the cage location corrected in ink.</t>
+          <t>DRF group</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Source reference</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Disposition</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Vehicle group</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>OQ/2010/000311: group animal-card file</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Individual card identifiers unavailable in this workbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Low-dose group</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>OQ/2010/000311: group animal-card file</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Individual card identifiers unavailable in this workbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Intermediate-dose group</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>OQ/2010/000311: group animal-card file</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Individual card identifiers unavailable in this workbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Top-dose group</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>OQ/2010/000311: group animal-card file</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Individual card identifiers unavailable in this workbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Top-dose reconciliation</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Group table is retained as the source summary. The individual card for the welfare intervention and its dose allocation are unavailable; complete individual reconciliation cannot be claimed.</t>
         </is>
       </c>
     </row>

</xml_diff>